<commit_message>
ajout detection des dependance inter feuilles , support feuilles sans header , plusieurs tableaux sur un  meme feuille et detection des erreurs
</commit_message>
<xml_diff>
--- a/data/excelphase3.1.xlsx
+++ b/data/excelphase3.1.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Documents\Excelium\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C548E0-2284-45EE-969E-EDAC36F1DAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6D2148-AFAD-4C7C-93CF-E8AAF8CFFF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2273" yWindow="1373" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="feuille1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>